<commit_message>
V4.3 | 2026.06.29 -CICD- 07/03/2026 10:38:53 AM
</commit_message>
<xml_diff>
--- a/Carga Masiva/detalle_reg_contable.xlsx
+++ b/Carga Masiva/detalle_reg_contable.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24334"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\benjfel\Desktop\CARGA REGISTROS CONTABLES\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\RepositoriosAEC\Acrux-Release\Carga Masiva\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F204DBA0-2CFA-4AC4-A582-4D99B593AA27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9192"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="detalle_reg_contable" sheetId="1" r:id="rId1"/>
@@ -19,12 +20,15 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="28">
   <si>
     <t>DEBITO</t>
   </si>
@@ -105,12 +109,15 @@
   </si>
   <si>
     <t>COD_ORDEN_CONTROL</t>
+  </si>
+  <si>
+    <t>DEPARTAMENTO</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -421,8 +428,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L5"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:M5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="7.21875" bestFit="1" customWidth="1"/>
@@ -437,9 +444,10 @@
     <col min="10" max="10" width="21" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="16.44140625" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="15.109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="25.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -476,8 +484,11 @@
       <c r="L1" t="s">
         <v>14</v>
       </c>
+      <c r="M1" t="s">
+        <v>27</v>
+      </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>500</v>
       </c>
@@ -515,7 +526,7 @@
         <v>1300</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>0</v>
       </c>
@@ -553,7 +564,7 @@
         <v>1762</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>2800</v>
       </c>
@@ -591,7 +602,7 @@
         <v>1250</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>0</v>
       </c>

</xml_diff>